<commit_message>
test(backend): add ORB icon matching assertion to brief upload test
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/test_brief.xlsx
+++ b/backend/tests/fixtures/test_brief.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="PL-PL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="COPY DECK" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -135,6 +122,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="952500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -426,96 +443,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A10:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>RATING</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>AGE</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>PEGI</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
-          <t>Hello</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Desc</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>World</t>
+          <t>18</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Hello</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Desc</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>World</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>